<commit_message>
Polish final CS13 submission and update README after merge
</commit_message>
<xml_diff>
--- a/Tennhombimat_CS13.xlsx
+++ b/Tennhombimat_CS13.xlsx
@@ -1254,7 +1254,7 @@
         <ns0:v>20</ns0:v>
       </ns0:c>
       <ns0:c r="E5" s="8" t="str">
-        <ns0:v>Tennhombimat | Nguyễn Anh Dũng | MSSV 2A202602554. Hồ sơ tr.6–7: 2.968 + 1.200 đ/bản, 15 triệu/1.200 bản. Rà soát hồ sơ có hỗ trợ AI, không phải xác nhận đã thử nghiệm.</ns0:v>
+        <ns0:v>Tennhombimat. Nguyễn Anh Dũng. MSSV 2A202602554. Hồ sơ tr.6–7: 2.968 + 1.200 đ/bản, 15 triệu/1.200 bản. Số liệu thuộc tình huống giả định.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="6" customFormat="false" ht="85" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1271,7 +1271,7 @@
         <ns0:v>23</ns0:v>
       </ns0:c>
       <ns0:c r="E6" s="8" t="str">
-        <ns0:v>Nhóm 1 người. Nguyễn Anh Dũng phụ trách CP0–CP5 với AI hỗ trợ soạn và kiểm tra. 1 việc = 1 bản nháp/1 người bệnh; BS bệnh viện ký 100%.</ns0:v>
+        <ns0:v>Nhóm một thành viên. Nguyễn Anh Dũng phụ trách CP0–CP5. Một việc = một bản nháp cho một người bệnh. BS bệnh viện đọc, sửa và ký 100%.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="7" customFormat="false" ht="85" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1288,7 +1288,7 @@
         <ns0:v>26</ns0:v>
       </ns0:c>
       <ns0:c r="E7" s="8" t="str">
-        <ns0:v>Giữ đủ 6 việc gợi ý. Điểm và ngưỡng mới là đề xuất để nhóm phản biện, chưa phải kết quả đo.</ns0:v>
+        <ns0:v>Đánh giá đủ sáu công việc gợi ý. Các ngưỡng bổ sung là mục tiêu kiểm chứng, chưa phải kết quả đo.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="8" customFormat="false" ht="85" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1322,7 +1322,7 @@
         <ns0:v>32</ns0:v>
       </ns0:c>
       <ns0:c r="E9" s="8" t="str">
-        <ns0:v>40 ca cần 20,3 giờ chuyên gia. Giả định lập kế hoạch: BS 2 giờ/tuần, DS 4 giờ/tuần; 5 ca insulin dự trù thêm 4 giờ tổng. Chưa có cam kết lịch thực tế.</ns0:v>
+        <ns0:v>40 ca cần 20,3 giờ chuyên gia. Giả định lập kế hoạch: BS chấm đánh giá 2 giờ/tuần, DS 4 giờ/tuần; 5 ca insulin dự trù thêm 4 giờ tổng. Lịch thực hiện xác nhận trước pilot.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="10" customFormat="false" ht="85" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1515,7 +1515,7 @@
         <ns0:v>Tự làm</ns0:v>
       </ns0:c>
       <ns0:c r="Q5" s="32" t="str">
-        <ns0:v>Có 40 hồ sơ nhưng chưa phát hành. Điểm sẵn sàng 0,8 phản ánh lỗi còn mở. Tích hợp và dẫn nguồn tạo giá trị; AI dự báo mô hình miễn phí dễ làm phần viết nháp, chưa kiểm chứng. Làm sau chặn lỗi thuốc.</ns0:v>
+        <ns0:v>Có 40 hồ sơ nhưng chưa phát hành; sẵn sàng 0,8 phản ánh lỗi còn mở. Giá trị nằm ở tích hợp và dẫn nguồn. Rủi ro thay thế L=0,5 do viết nháp có thể thành chức năng phổ biến; đây là giả định chiến lược. Triển khai sau chặn lỗi thuốc.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="6" customFormat="false" ht="145" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1571,7 +1571,7 @@
         <ns0:v>Tự làm</ns0:v>
       </ns0:c>
       <ns0:c r="Q6" s="32" t="str">
-        <ns0:v>Ưu tiên an toàn bắt buộc: lỗi insulin sáng/tối đã xảy ra. Bộ đề sẵn có, cần 5 ca bổ sung. L=0,2 là nhận định AI: kiểm chứng theo y lệnh và quy trình địa phương khó thay bằng chức năng chung. Không coi dự báo là bằng chứng.</ns0:v>
+        <ns0:v>Ưu tiên an toàn: đã có lỗi insulin sáng/tối. Bộ đề cần bổ sung 5 ca. L=0,2 vì đối chiếu y lệnh và kiểm chứng quy trình địa phương khó thay bằng chức năng chung. Chỉ mở pilot sau cổng hồi quy.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="7" customFormat="false" ht="145" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1627,7 +1627,7 @@
         <ns0:v>Tự làm</ns0:v>
       </ns0:c>
       <ns0:c r="Q7" s="32" t="str">
-        <ns0:v>40 ca có 4 tầng nhưng số ca mâu thuẫn chưa rõ nên J/K=0,7. Ưu tiên trước nháp đại trà dù điểm có thể gần nhau. L=0,3 do cần nối hồ sơ và kiểm chứng nguồn. Ngưỡng/cỡ mẫu mới đều là đề xuất.</ns0:v>
+        <ns0:v>Bộ 40 ca có bốn tầng nhưng chưa rõ số ca mâu thuẫn, nên J/K=0,7. Ưu tiên trước nháp đại trà theo điều kiện an toàn. L=0,3 do cần kết nối và kiểm chứng nguồn. Ngưỡng/cỡ mẫu bổ sung là đề xuất.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="8" customFormat="false" ht="145" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1683,7 +1683,7 @@
         <ns0:v>Chờ</ns0:v>
       </ns0:c>
       <ns0:c r="Q8" s="32" t="str">
-        <ns0:v>AI dự báo diễn đạt dễ hiểu có thể thành tính năng miễn phí (L=0,9), nhưng hiểu và tuân thủ cần kiểm chứng. Chưa có bộ đánh giá riêng nên K=0,3. Xem lại tháng 6 sau khi nháp cốt lõi an toàn; chưa tuyên bố cải thiện tuân thủ thật.</ns0:v>
+        <ns0:v>Diễn đạt dễ hiểu có thể trở thành chức năng phổ biến (L=0,9), nhưng khả năng hiểu và tuân thủ cần kiểm chứng. Chưa có bộ đánh giá riêng nên K=0,3. Xem lại tháng 6 sau khi nháp cốt lõi an toàn.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="9" customFormat="false" ht="145" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -1739,7 +1739,7 @@
         <ns0:v>Chờ</ns0:v>
       </ns0:c>
       <ns0:c r="Q9" s="32" t="str">
-        <ns0:v>Hồ sơ nói chưa có bộ đề chuyển khoa. J=0,3, K=0,1 do khác phạm vi. Chỉ khám phá tháng 6–12 sau hợp đồng và cổng riêng; không dùng 45 ca ra viện để phê duyệt. L=0,4 là dự báo AI cần xem lại.</ns0:v>
+        <ns0:v>Chưa có bộ đề chuyển khoa. J=0,3, K=0,1 do khác phạm vi ra viện. Khám phá tháng 6–12 sau hợp đồng và cổng riêng; không dùng 45 ca ra viện để phê duyệt. L=0,4 là ước lượng chiến lược cần xem lại.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="10" customFormat="false" ht="145" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
@@ -3022,7 +3022,7 @@
     <ns0:row r="12" customFormat="false" ht="60" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
       <ns0:c r="A12" s="9"/>
       <ns0:c r="D12" s="28" t="str">
-        <ns0:v>Tự chấm AI: 94/100 (tham khảo).</ns0:v>
+        <ns0:v>Tự chấm: 94/100 (tham khảo).</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Remove self grading from final submission
</commit_message>
<xml_diff>
--- a/Tennhombimat_CS13.xlsx
+++ b/Tennhombimat_CS13.xlsx
@@ -2946,9 +2946,7 @@
       <ns0:c r="C5" s="27" t="s">
         <ns0:v>152</ns0:v>
       </ns0:c>
-      <ns0:c r="D5" s="28" t="n">
-        <ns0:v>19</ns0:v>
-      </ns0:c>
+      <ns0:c r="D5" s="28"/>
     </ns0:row>
     <ns0:row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A6" s="11" t="s">
@@ -2960,9 +2958,7 @@
       <ns0:c r="C6" s="27" t="s">
         <ns0:v>154</ns0:v>
       </ns0:c>
-      <ns0:c r="D6" s="28" t="n">
-        <ns0:v>19</ns0:v>
-      </ns0:c>
+      <ns0:c r="D6" s="28"/>
     </ns0:row>
     <ns0:row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A7" s="11" t="s">
@@ -2974,9 +2970,7 @@
       <ns0:c r="C7" s="27" t="s">
         <ns0:v>156</ns0:v>
       </ns0:c>
-      <ns0:c r="D7" s="28" t="n">
-        <ns0:v>23</ns0:v>
-      </ns0:c>
+      <ns0:c r="D7" s="28"/>
     </ns0:row>
     <ns0:row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A8" s="11" t="s">
@@ -2988,9 +2982,7 @@
       <ns0:c r="C8" s="27" t="s">
         <ns0:v>158</ns0:v>
       </ns0:c>
-      <ns0:c r="D8" s="28" t="n">
-        <ns0:v>14</ns0:v>
-      </ns0:c>
+      <ns0:c r="D8" s="28"/>
     </ns0:row>
     <ns0:row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A9" s="11" t="s">
@@ -3002,9 +2994,7 @@
       <ns0:c r="C9" s="27" t="s">
         <ns0:v>160</ns0:v>
       </ns0:c>
-      <ns0:c r="D9" s="28" t="n">
-        <ns0:v>19</ns0:v>
-      </ns0:c>
+      <ns0:c r="D9" s="28"/>
     </ns0:row>
     <ns0:row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A10" s="9" t="s">
@@ -3016,14 +3006,12 @@
       </ns0:c>
       <ns0:c r="D10" s="12" t="n">
         <ns0:f aca="false">SUM(D5:D9)</ns0:f>
-        <ns0:v>94</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="12" customFormat="false" ht="60" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
       <ns0:c r="A12" s="9"/>
-      <ns0:c r="D12" s="28" t="str">
-        <ns0:v>Tự chấm: 94/100 (tham khảo).</ns0:v>
-      </ns0:c>
+      <ns0:c r="D12" s="28"/>
     </ns0:row>
     <ns0:row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <ns0:c r="A15" s="29" t="s">

</xml_diff>